<commit_message>
Aligne les couleurs du calendrier sur la charte graphique du site
Remplace la palette bleu/violet/vert par les couleurs de marque
(teal, orange, teal foncé, anthracite) issues de brand-book.html,
avec un titre en Georgia pour rappeler le Playfair Display du site.
</commit_message>
<xml_diff>
--- a/Calendrier_Rituels_Manager.xlsx
+++ b/Calendrier_Rituels_Manager.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -142,8 +142,77 @@
       <color rgb="FFFFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Georgia"/>
+      <color rgb="FFFDF8F3"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF0A5F62"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFDF8F3"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <i val="1"/>
+      <color rgb="FFFDF8F3"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF0F868A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF3A352F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF0A5F62"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFF914D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF8A8378"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF2D2D2D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFE8792A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <i val="1"/>
+      <color rgb="FFFDF8F3"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="29">
     <fill>
       <patternFill/>
     </fill>
@@ -241,8 +310,63 @@
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDF8F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2D2D2D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF8F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0F868A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF914D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF1E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0A5F62"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCFE9E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F1EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8792A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE8D6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="14">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -424,6 +548,238 @@
         <color rgb="000F868A"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000F868A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000F868A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9CEC0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9CEC0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9CEC0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9CEC0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000F868A"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="000F868A"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="000F868A"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000F868A"/>
+      </right>
+      <top style="medium">
+        <color rgb="000F868A"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000F868A"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000F868A"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000F868A"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9CEC0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9CEC0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9CEC0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9CEC0"/>
+      </left>
+      <right style="medium">
+        <color rgb="000F868A"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9CEC0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9CEC0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000F868A"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000F868A"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000F868A"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000F868A"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000F868A"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="000F868A"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="000F868A"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="000F868A"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="000F868A"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -435,7 +791,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="139">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -652,6 +1008,141 @@
     <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="19" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -906,7 +1397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:G36"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="27" min="1" max="1"/>
@@ -920,781 +1411,876 @@
   </cols>
   <sheetData>
     <row r="1" ht="39.75" customHeight="1" s="28">
-      <c r="B1" s="29" t="inlineStr">
+      <c r="A1" s="76" t="n"/>
+      <c r="B1" s="77" t="inlineStr">
         <is>
           <t>📆 CALENDRIER DES RITUELS MANAGÉRIAUX — Septembre à Décembre 2026</t>
         </is>
       </c>
+      <c r="C1" s="78" t="n"/>
+      <c r="D1" s="78" t="n"/>
+      <c r="E1" s="78" t="n"/>
+      <c r="F1" s="78" t="n"/>
+      <c r="G1" s="79" t="n"/>
+      <c r="H1" s="76" t="n"/>
     </row>
     <row r="2" ht="21.75" customHeight="1" s="28">
-      <c r="B2" s="30" t="inlineStr">
-        <is>
-          <t>Quotidien (teal) · Hebdomadaire (orange) · Mensuel (bleu) · Trimestriel/Ponctuel (violet) · Rentrée (vert)</t>
-        </is>
-      </c>
+      <c r="A2" s="76" t="n"/>
+      <c r="B2" s="80" t="inlineStr">
+        <is>
+          <t>Quotidien (teal) · Hebdomadaire (orange) · Mensuel (teal foncé) · Trimestriel/Ponctuel (anthracite) · Rentrée (orange foncé)</t>
+        </is>
+      </c>
+      <c r="C2" s="81" t="n"/>
+      <c r="D2" s="81" t="n"/>
+      <c r="E2" s="81" t="n"/>
+      <c r="F2" s="81" t="n"/>
+      <c r="G2" s="82" t="n"/>
+      <c r="H2" s="76" t="n"/>
     </row>
     <row r="3" ht="25.5" customHeight="1" s="28">
-      <c r="B3" s="31" t="inlineStr">
+      <c r="A3" s="76" t="n"/>
+      <c r="B3" s="83" t="inlineStr">
         <is>
           <t>Fréquence</t>
         </is>
       </c>
-      <c r="C3" s="32" t="inlineStr">
+      <c r="C3" s="84" t="inlineStr">
         <is>
           <t>Rituel</t>
         </is>
       </c>
-      <c r="D3" s="32" t="inlineStr">
+      <c r="D3" s="84" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="E3" s="32" t="inlineStr">
+      <c r="E3" s="84" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="F3" s="32" t="inlineStr">
+      <c r="F3" s="84" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="G3" s="33" t="inlineStr">
+      <c r="G3" s="85" t="inlineStr">
         <is>
           <t>Déc</t>
         </is>
       </c>
+      <c r="H3" s="76" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1" s="28">
-      <c r="B4" s="34" t="inlineStr">
+      <c r="A4" s="76" t="n"/>
+      <c r="B4" s="86" t="inlineStr">
         <is>
           <t>── QUOTIDIEN ──</t>
         </is>
       </c>
-      <c r="C4" s="35" t="n"/>
-      <c r="D4" s="35" t="n"/>
-      <c r="E4" s="35" t="n"/>
-      <c r="F4" s="35" t="n"/>
-      <c r="G4" s="36" t="n"/>
+      <c r="C4" s="87" t="n"/>
+      <c r="D4" s="87" t="n"/>
+      <c r="E4" s="87" t="n"/>
+      <c r="F4" s="87" t="n"/>
+      <c r="G4" s="88" t="n"/>
+      <c r="H4" s="76" t="n"/>
     </row>
     <row r="5" ht="36" customHeight="1" s="28">
-      <c r="B5" s="37" t="inlineStr">
+      <c r="A5" s="76" t="n"/>
+      <c r="B5" s="89" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C5" s="38" t="inlineStr">
+      <c r="C5" s="90" t="inlineStr">
         <is>
           <t>Morning brief
 Chaque jour — 10 min avant les mails</t>
         </is>
       </c>
-      <c r="D5" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E5" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F5" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G5" s="40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D5" s="91" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E5" s="91" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F5" s="91" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G5" s="92" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H5" s="76" t="n"/>
     </row>
     <row r="6" ht="7.5" customHeight="1" s="28">
-      <c r="B6" s="41" t="n"/>
-      <c r="C6" s="35" t="n"/>
-      <c r="D6" s="35" t="n"/>
-      <c r="E6" s="35" t="n"/>
-      <c r="F6" s="35" t="n"/>
-      <c r="G6" s="36" t="n"/>
+      <c r="A6" s="76" t="n"/>
+      <c r="B6" s="93" t="n"/>
+      <c r="C6" s="94" t="n"/>
+      <c r="D6" s="94" t="n"/>
+      <c r="E6" s="94" t="n"/>
+      <c r="F6" s="94" t="n"/>
+      <c r="G6" s="95" t="n"/>
+      <c r="H6" s="76" t="n"/>
     </row>
     <row r="7" ht="24" customHeight="1" s="28">
-      <c r="B7" s="42" t="inlineStr">
+      <c r="A7" s="76" t="n"/>
+      <c r="B7" s="96" t="inlineStr">
         <is>
           <t>── HEBDOMADAIRE ──</t>
         </is>
       </c>
-      <c r="C7" s="35" t="n"/>
-      <c r="D7" s="35" t="n"/>
-      <c r="E7" s="35" t="n"/>
-      <c r="F7" s="35" t="n"/>
-      <c r="G7" s="36" t="n"/>
+      <c r="C7" s="97" t="n"/>
+      <c r="D7" s="97" t="n"/>
+      <c r="E7" s="97" t="n"/>
+      <c r="F7" s="97" t="n"/>
+      <c r="G7" s="98" t="n"/>
+      <c r="H7" s="76" t="n"/>
     </row>
     <row r="8" ht="36" customHeight="1" s="28">
-      <c r="B8" s="43" t="inlineStr">
+      <c r="A8" s="76" t="n"/>
+      <c r="B8" s="99" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C8" s="44" t="inlineStr">
+      <c r="C8" s="100" t="inlineStr">
         <is>
           <t>OTO collaborateurs
 Chaque semaine — 30 min/personne</t>
         </is>
       </c>
-      <c r="D8" s="45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E8" s="45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F8" s="45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G8" s="46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D8" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E8" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F8" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G8" s="102" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H8" s="76" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1" s="28">
-      <c r="B9" s="47" t="inlineStr">
+      <c r="A9" s="76" t="n"/>
+      <c r="B9" s="99" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C9" s="48" t="inlineStr">
+      <c r="C9" s="100" t="inlineStr">
         <is>
           <t>Réunion d'équipe hebdo
 Ordre du jour + Qui/Quoi/Pour quand</t>
         </is>
       </c>
-      <c r="D9" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E9" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F9" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G9" s="40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D9" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E9" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F9" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G9" s="102" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H9" s="76" t="n"/>
     </row>
     <row r="10" ht="36" customHeight="1" s="28">
-      <c r="B10" s="43" t="inlineStr">
+      <c r="A10" s="76" t="n"/>
+      <c r="B10" s="99" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C10" s="44" t="inlineStr">
+      <c r="C10" s="100" t="inlineStr">
         <is>
           <t>Bilan du vendredi
 10 min — finir l'esprit léger</t>
         </is>
       </c>
-      <c r="D10" s="45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E10" s="45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F10" s="45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G10" s="46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D10" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E10" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F10" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G10" s="102" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H10" s="76" t="n"/>
     </row>
     <row r="11" ht="36" customHeight="1" s="28">
-      <c r="B11" s="47" t="inlineStr">
+      <c r="A11" s="76" t="n"/>
+      <c r="B11" s="99" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C11" s="48" t="inlineStr">
+      <c r="C11" s="100" t="inlineStr">
         <is>
           <t>Stratégie managériale ✦
 Toutes les 2 semaines — 1h seul</t>
         </is>
       </c>
-      <c r="D11" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E11" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F11" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G11" s="40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D11" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E11" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F11" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G11" s="102" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H11" s="76" t="n"/>
     </row>
     <row r="12" ht="36" customHeight="1" s="28">
-      <c r="B12" s="43" t="inlineStr">
+      <c r="A12" s="76" t="n"/>
+      <c r="B12" s="99" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C12" s="44" t="inlineStr">
+      <c r="C12" s="100" t="inlineStr">
         <is>
           <t>OTO départ en congés
 Avant chaque départ — cadrer passation</t>
         </is>
       </c>
-      <c r="D12" s="49" t="inlineStr">
+      <c r="D12" s="103" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="49" t="inlineStr">
+      <c r="E12" s="103" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F12" s="45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G12" s="46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F12" s="101" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G12" s="102" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H12" s="76" t="n"/>
     </row>
     <row r="13" ht="7.5" customHeight="1" s="28">
-      <c r="B13" s="41" t="n"/>
-      <c r="C13" s="35" t="n"/>
-      <c r="D13" s="35" t="n"/>
-      <c r="E13" s="35" t="n"/>
-      <c r="F13" s="35" t="n"/>
-      <c r="G13" s="36" t="n"/>
+      <c r="A13" s="76" t="n"/>
+      <c r="B13" s="93" t="n"/>
+      <c r="C13" s="94" t="n"/>
+      <c r="D13" s="94" t="n"/>
+      <c r="E13" s="94" t="n"/>
+      <c r="F13" s="94" t="n"/>
+      <c r="G13" s="95" t="n"/>
+      <c r="H13" s="76" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1" s="28">
-      <c r="B14" s="50" t="inlineStr">
+      <c r="A14" s="76" t="n"/>
+      <c r="B14" s="104" t="inlineStr">
         <is>
           <t>── MENSUEL ──</t>
         </is>
       </c>
-      <c r="C14" s="35" t="n"/>
-      <c r="D14" s="35" t="n"/>
-      <c r="E14" s="35" t="n"/>
-      <c r="F14" s="35" t="n"/>
-      <c r="G14" s="36" t="n"/>
+      <c r="C14" s="105" t="n"/>
+      <c r="D14" s="105" t="n"/>
+      <c r="E14" s="105" t="n"/>
+      <c r="F14" s="105" t="n"/>
+      <c r="G14" s="106" t="n"/>
+      <c r="H14" s="76" t="n"/>
     </row>
     <row r="15" ht="36" customHeight="1" s="28">
-      <c r="B15" s="51" t="inlineStr">
+      <c r="A15" s="76" t="n"/>
+      <c r="B15" s="107" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C15" s="52" t="inlineStr">
+      <c r="C15" s="108" t="inlineStr">
         <is>
           <t>Revue de performance individuelle
 S3 de chaque mois</t>
         </is>
       </c>
-      <c r="D15" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E15" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F15" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G15" s="40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D15" s="109" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E15" s="109" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F15" s="109" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G15" s="110" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H15" s="76" t="n"/>
     </row>
     <row r="16" ht="36" customHeight="1" s="28">
-      <c r="B16" s="53" t="inlineStr">
+      <c r="A16" s="76" t="n"/>
+      <c r="B16" s="107" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C16" s="54" t="inlineStr">
+      <c r="C16" s="108" t="inlineStr">
         <is>
           <t>Rétrospective équipe
 S3 de chaque mois</t>
         </is>
       </c>
-      <c r="D16" s="45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E16" s="45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F16" s="45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G16" s="46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D16" s="109" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E16" s="109" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F16" s="109" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G16" s="110" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H16" s="76" t="n"/>
     </row>
     <row r="17" ht="36" customHeight="1" s="28">
-      <c r="B17" s="51" t="inlineStr">
+      <c r="A17" s="76" t="n"/>
+      <c r="B17" s="107" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C17" s="52" t="inlineStr">
+      <c r="C17" s="108" t="inlineStr">
         <is>
           <t>Point avec mon N+1
 S3 de chaque mois</t>
         </is>
       </c>
-      <c r="D17" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E17" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F17" s="39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G17" s="40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D17" s="109" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E17" s="109" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F17" s="109" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G17" s="110" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H17" s="76" t="n"/>
     </row>
     <row r="18" ht="7.5" customHeight="1" s="28">
-      <c r="B18" s="41" t="n"/>
-      <c r="C18" s="35" t="n"/>
-      <c r="D18" s="35" t="n"/>
-      <c r="E18" s="35" t="n"/>
-      <c r="F18" s="35" t="n"/>
-      <c r="G18" s="36" t="n"/>
+      <c r="A18" s="76" t="n"/>
+      <c r="B18" s="93" t="n"/>
+      <c r="C18" s="94" t="n"/>
+      <c r="D18" s="94" t="n"/>
+      <c r="E18" s="94" t="n"/>
+      <c r="F18" s="94" t="n"/>
+      <c r="G18" s="95" t="n"/>
+      <c r="H18" s="76" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1" s="28">
-      <c r="B19" s="55" t="inlineStr">
+      <c r="A19" s="76" t="n"/>
+      <c r="B19" s="111" t="inlineStr">
         <is>
           <t>── TRIMESTRIEL ──</t>
         </is>
       </c>
-      <c r="C19" s="35" t="n"/>
-      <c r="D19" s="35" t="n"/>
-      <c r="E19" s="35" t="n"/>
-      <c r="F19" s="35" t="n"/>
-      <c r="G19" s="36" t="n"/>
+      <c r="C19" s="112" t="n"/>
+      <c r="D19" s="112" t="n"/>
+      <c r="E19" s="112" t="n"/>
+      <c r="F19" s="112" t="n"/>
+      <c r="G19" s="113" t="n"/>
+      <c r="H19" s="76" t="n"/>
     </row>
     <row r="20" ht="36" customHeight="1" s="28">
-      <c r="B20" s="56" t="inlineStr">
+      <c r="A20" s="76" t="n"/>
+      <c r="B20" s="114" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="C20" s="57" t="inlineStr">
+      <c r="C20" s="115" t="inlineStr">
         <is>
           <t>Revue des objectifs
 Fin de trimestre</t>
         </is>
       </c>
-      <c r="D20" s="45" t="inlineStr">
+      <c r="D20" s="116" t="inlineStr">
         <is>
           <t>✅ fin sept</t>
         </is>
       </c>
-      <c r="E20" s="58" t="inlineStr">
+      <c r="E20" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F20" s="58" t="inlineStr">
+      <c r="F20" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G20" s="46" t="inlineStr">
+      <c r="G20" s="118" t="inlineStr">
         <is>
           <t>✅ fin déc</t>
         </is>
       </c>
+      <c r="H20" s="76" t="n"/>
     </row>
     <row r="21" ht="36" customHeight="1" s="28">
-      <c r="B21" s="59" t="inlineStr">
+      <c r="A21" s="76" t="n"/>
+      <c r="B21" s="114" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="C21" s="60" t="inlineStr">
+      <c r="C21" s="115" t="inlineStr">
         <is>
           <t>Bilan managérial
 Fin de trimestre</t>
         </is>
       </c>
-      <c r="D21" s="39" t="inlineStr">
+      <c r="D21" s="116" t="inlineStr">
         <is>
           <t>✅ fin sept</t>
         </is>
       </c>
-      <c r="E21" s="61" t="inlineStr">
+      <c r="E21" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F21" s="61" t="inlineStr">
+      <c r="F21" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G21" s="40" t="inlineStr">
+      <c r="G21" s="118" t="inlineStr">
         <is>
           <t>✅ fin déc</t>
         </is>
       </c>
+      <c r="H21" s="76" t="n"/>
     </row>
     <row r="22" ht="36" customHeight="1" s="28">
-      <c r="B22" s="56" t="inlineStr">
+      <c r="A22" s="76" t="n"/>
+      <c r="B22" s="114" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="C22" s="57" t="inlineStr">
+      <c r="C22" s="115" t="inlineStr">
         <is>
           <t>Feedback ascendant
 1 question simple à l'équipe</t>
         </is>
       </c>
-      <c r="D22" s="45" t="inlineStr">
+      <c r="D22" s="116" t="inlineStr">
         <is>
           <t>✅ fin sept</t>
         </is>
       </c>
-      <c r="E22" s="58" t="inlineStr">
+      <c r="E22" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F22" s="58" t="inlineStr">
+      <c r="F22" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G22" s="46" t="inlineStr">
+      <c r="G22" s="118" t="inlineStr">
         <is>
           <t>✅ mi-déc</t>
         </is>
       </c>
+      <c r="H22" s="76" t="n"/>
     </row>
     <row r="23" ht="7.5" customHeight="1" s="28">
-      <c r="B23" s="41" t="n"/>
-      <c r="C23" s="35" t="n"/>
-      <c r="D23" s="35" t="n"/>
-      <c r="E23" s="35" t="n"/>
-      <c r="F23" s="35" t="n"/>
-      <c r="G23" s="36" t="n"/>
+      <c r="A23" s="76" t="n"/>
+      <c r="B23" s="93" t="n"/>
+      <c r="C23" s="94" t="n"/>
+      <c r="D23" s="94" t="n"/>
+      <c r="E23" s="94" t="n"/>
+      <c r="F23" s="94" t="n"/>
+      <c r="G23" s="95" t="n"/>
+      <c r="H23" s="76" t="n"/>
     </row>
     <row r="24" ht="24" customHeight="1" s="28">
-      <c r="B24" s="55" t="inlineStr">
+      <c r="A24" s="76" t="n"/>
+      <c r="B24" s="111" t="inlineStr">
         <is>
           <t>── PONCTUEL ──</t>
         </is>
       </c>
-      <c r="C24" s="35" t="n"/>
-      <c r="D24" s="35" t="n"/>
-      <c r="E24" s="35" t="n"/>
-      <c r="F24" s="35" t="n"/>
-      <c r="G24" s="36" t="n"/>
+      <c r="C24" s="112" t="n"/>
+      <c r="D24" s="112" t="n"/>
+      <c r="E24" s="112" t="n"/>
+      <c r="F24" s="112" t="n"/>
+      <c r="G24" s="113" t="n"/>
+      <c r="H24" s="76" t="n"/>
     </row>
     <row r="25" ht="36" customHeight="1" s="28">
-      <c r="B25" s="59" t="inlineStr">
+      <c r="A25" s="76" t="n"/>
+      <c r="B25" s="114" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="C25" s="60" t="inlineStr">
+      <c r="C25" s="115" t="inlineStr">
         <is>
           <t>Préparer entretiens professionnels
 Planifier, collecter les éléments</t>
         </is>
       </c>
-      <c r="D25" s="61" t="inlineStr">
+      <c r="D25" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E25" s="39" t="inlineStr">
+      <c r="E25" s="116" t="inlineStr">
         <is>
           <t>✅ mi-oct</t>
         </is>
       </c>
-      <c r="F25" s="61" t="inlineStr">
+      <c r="F25" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G25" s="62" t="inlineStr">
+      <c r="G25" s="119" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="H25" s="76" t="n"/>
     </row>
     <row r="26" ht="36" customHeight="1" s="28">
-      <c r="B26" s="56" t="inlineStr">
+      <c r="A26" s="76" t="n"/>
+      <c r="B26" s="114" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="C26" s="57" t="inlineStr">
+      <c r="C26" s="115" t="inlineStr">
         <is>
           <t>Préparer entretiens annuels
 Grille, objectifs, bilan de l'année</t>
         </is>
       </c>
-      <c r="D26" s="58" t="inlineStr">
+      <c r="D26" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E26" s="58" t="inlineStr">
+      <c r="E26" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F26" s="45" t="inlineStr">
+      <c r="F26" s="116" t="inlineStr">
         <is>
           <t>✅ mi-nov</t>
         </is>
       </c>
-      <c r="G26" s="46" t="inlineStr">
+      <c r="G26" s="118" t="inlineStr">
         <is>
           <t>✅ début déc</t>
         </is>
       </c>
+      <c r="H26" s="76" t="n"/>
     </row>
     <row r="27" ht="36" customHeight="1" s="28">
-      <c r="B27" s="59" t="inlineStr">
+      <c r="A27" s="76" t="n"/>
+      <c r="B27" s="114" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="C27" s="60" t="inlineStr">
+      <c r="C27" s="115" t="inlineStr">
         <is>
           <t>Célébration victoires équipe
 Avant les fêtes — reconnaître les accomplissements</t>
         </is>
       </c>
-      <c r="D27" s="61" t="inlineStr">
+      <c r="D27" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E27" s="61" t="inlineStr">
+      <c r="E27" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F27" s="61" t="inlineStr">
+      <c r="F27" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G27" s="40" t="inlineStr">
+      <c r="G27" s="118" t="inlineStr">
         <is>
           <t>✅ mi-déc</t>
         </is>
       </c>
+      <c r="H27" s="76" t="n"/>
     </row>
     <row r="28" ht="36" customHeight="1" s="28">
-      <c r="B28" s="56" t="inlineStr">
+      <c r="A28" s="76" t="n"/>
+      <c r="B28" s="114" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="C28" s="57" t="inlineStr">
+      <c r="C28" s="115" t="inlineStr">
         <is>
           <t>Voeux et clôture de l'année
 Rituel collectif — cap de l'année qui vient</t>
         </is>
       </c>
-      <c r="D28" s="58" t="inlineStr">
+      <c r="D28" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E28" s="58" t="inlineStr">
+      <c r="E28" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F28" s="58" t="inlineStr">
+      <c r="F28" s="117" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G28" s="46" t="inlineStr">
+      <c r="G28" s="118" t="inlineStr">
         <is>
           <t>✅ fin déc</t>
         </is>
       </c>
+      <c r="H28" s="76" t="n"/>
     </row>
     <row r="29" ht="7.5" customHeight="1" s="28">
-      <c r="B29" s="41" t="n"/>
-      <c r="C29" s="35" t="n"/>
-      <c r="D29" s="35" t="n"/>
-      <c r="E29" s="35" t="n"/>
-      <c r="F29" s="35" t="n"/>
-      <c r="G29" s="36" t="n"/>
+      <c r="A29" s="76" t="n"/>
+      <c r="B29" s="93" t="n"/>
+      <c r="C29" s="94" t="n"/>
+      <c r="D29" s="94" t="n"/>
+      <c r="E29" s="94" t="n"/>
+      <c r="F29" s="94" t="n"/>
+      <c r="G29" s="95" t="n"/>
+      <c r="H29" s="76" t="n"/>
     </row>
     <row r="30" ht="27.75" customHeight="1" s="28">
-      <c r="B30" s="63" t="inlineStr">
+      <c r="A30" s="76" t="n"/>
+      <c r="B30" s="120" t="inlineStr">
         <is>
           <t>🎒 RENTRÉE SPÉCIALE — Septembre uniquement</t>
         </is>
       </c>
-      <c r="C30" s="35" t="n"/>
-      <c r="D30" s="35" t="n"/>
-      <c r="E30" s="35" t="n"/>
-      <c r="F30" s="35" t="n"/>
-      <c r="G30" s="36" t="n"/>
+      <c r="C30" s="121" t="n"/>
+      <c r="D30" s="121" t="n"/>
+      <c r="E30" s="121" t="n"/>
+      <c r="F30" s="121" t="n"/>
+      <c r="G30" s="122" t="n"/>
+      <c r="H30" s="76" t="n"/>
     </row>
     <row r="31" ht="31.5" customHeight="1" s="28">
-      <c r="B31" s="64" t="inlineStr">
+      <c r="A31" s="76" t="n"/>
+      <c r="B31" s="123" t="inlineStr">
         <is>
           <t>🎒</t>
         </is>
       </c>
-      <c r="C31" s="65" t="inlineStr">
+      <c r="C31" s="124" t="inlineStr">
         <is>
           <t>1:1 de reprise avec chaque collaborateur
 S1 à S3 de septembre — comment il/elle revient</t>
         </is>
       </c>
-      <c r="D31" s="66" t="inlineStr">
+      <c r="D31" s="125" t="inlineStr">
         <is>
           <t>✅ Septembre uniquement</t>
         </is>
       </c>
-      <c r="E31" s="35" t="n"/>
-      <c r="F31" s="35" t="n"/>
-      <c r="G31" s="36" t="n"/>
+      <c r="E31" s="126" t="n"/>
+      <c r="F31" s="126" t="n"/>
+      <c r="G31" s="127" t="n"/>
+      <c r="H31" s="76" t="n"/>
     </row>
     <row r="32" ht="31.5" customHeight="1" s="28">
-      <c r="B32" s="67" t="inlineStr">
+      <c r="A32" s="76" t="n"/>
+      <c r="B32" s="123" t="inlineStr">
         <is>
           <t>🎒</t>
         </is>
       </c>
-      <c r="C32" s="68" t="inlineStr">
+      <c r="C32" s="124" t="inlineStr">
         <is>
           <t>Réunion de rentrée
 S1 ou S2 — 6 étapes, trame complète dans Notion</t>
         </is>
       </c>
-      <c r="D32" s="69" t="inlineStr">
+      <c r="D32" s="125" t="inlineStr">
         <is>
           <t>✅ Septembre uniquement</t>
         </is>
       </c>
-      <c r="E32" s="35" t="n"/>
-      <c r="F32" s="35" t="n"/>
-      <c r="G32" s="36" t="n"/>
+      <c r="E32" s="126" t="n"/>
+      <c r="F32" s="126" t="n"/>
+      <c r="G32" s="127" t="n"/>
+      <c r="H32" s="76" t="n"/>
     </row>
     <row r="33" ht="31.5" customHeight="1" s="28">
-      <c r="B33" s="64" t="inlineStr">
+      <c r="A33" s="76" t="n"/>
+      <c r="B33" s="123" t="inlineStr">
         <is>
           <t>🎒</t>
         </is>
       </c>
-      <c r="C33" s="65" t="inlineStr">
+      <c r="C33" s="124" t="inlineStr">
         <is>
           <t>Challenge de rentrée
 20 questions à poser avant le 30 septembre</t>
         </is>
       </c>
-      <c r="D33" s="66" t="inlineStr">
+      <c r="D33" s="125" t="inlineStr">
         <is>
           <t>✅ Septembre uniquement</t>
         </is>
       </c>
-      <c r="E33" s="35" t="n"/>
-      <c r="F33" s="35" t="n"/>
-      <c r="G33" s="36" t="n"/>
+      <c r="E33" s="126" t="n"/>
+      <c r="F33" s="126" t="n"/>
+      <c r="G33" s="127" t="n"/>
+      <c r="H33" s="76" t="n"/>
     </row>
     <row r="34" ht="31.5" customHeight="1" s="28">
-      <c r="B34" s="70" t="inlineStr">
+      <c r="A34" s="76" t="n"/>
+      <c r="B34" s="128" t="inlineStr">
         <is>
           <t>🎒</t>
         </is>
       </c>
-      <c r="C34" s="71" t="inlineStr">
+      <c r="C34" s="129" t="inlineStr">
         <is>
           <t>Checklist managériale de rentrée
 Tout ce qu'il faut avoir fait avant le 30 sept</t>
         </is>
       </c>
-      <c r="D34" s="72" t="inlineStr">
+      <c r="D34" s="130" t="inlineStr">
         <is>
           <t>✅ Septembre uniquement</t>
         </is>
       </c>
-      <c r="E34" s="73" t="n"/>
-      <c r="F34" s="73" t="n"/>
-      <c r="G34" s="74" t="n"/>
+      <c r="E34" s="131" t="n"/>
+      <c r="F34" s="131" t="n"/>
+      <c r="G34" s="132" t="n"/>
+      <c r="H34" s="76" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="76" t="n"/>
+      <c r="B35" s="133" t="n"/>
+      <c r="C35" s="134" t="n"/>
+      <c r="D35" s="134" t="n"/>
+      <c r="E35" s="134" t="n"/>
+      <c r="F35" s="134" t="n"/>
+      <c r="G35" s="135" t="n"/>
+      <c r="H35" s="76" t="n"/>
     </row>
     <row r="36" ht="25.5" customHeight="1" s="28">
-      <c r="B36" s="75" t="inlineStr">
+      <c r="A36" s="76" t="n"/>
+      <c r="B36" s="136" t="inlineStr">
         <is>
           <t>Le Cartable du Manager — Rentrée 2026 · Élodie Boyer · EB Formation Consulting</t>
         </is>
       </c>
+      <c r="C36" s="137" t="n"/>
+      <c r="D36" s="137" t="n"/>
+      <c r="E36" s="137" t="n"/>
+      <c r="F36" s="137" t="n"/>
+      <c r="G36" s="138" t="n"/>
+      <c r="H36" s="76" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">

</xml_diff>

<commit_message>
Retire le noir/anthracite du calendrier au profit de la palette officielle
Remplace toutes les couleurs sombres (titre, en-têtes, bandeaux
Trimestriel/Ponctuel) par des teintes tirées de palette_optp.html :
teal foncé (#085055) et orange foncé (#CC6A2E) à la place du noir,
et réattribue une couleur distincte par section sans doublon.
</commit_message>
<xml_diff>
--- a/Calendrier_Rituels_Manager.xlsx
+++ b/Calendrier_Rituels_Manager.xlsx
@@ -36,7 +36,7 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="FF0A5F62"/>
+      <color rgb="FF085055"/>
       <sz val="9"/>
     </font>
     <font>
@@ -65,13 +65,13 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="FF3A352F"/>
+      <color rgb="FF085055"/>
       <sz val="8.5"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="FF0A5F62"/>
+      <color rgb="FF085055"/>
       <sz val="10"/>
     </font>
     <font>
@@ -82,25 +82,25 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="FF8A8378"/>
+      <color rgb="FF6B9AA0"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="FF0A5F62"/>
+      <color rgb="FF085055"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="FF2D2D2D"/>
+      <color rgb="FFCC6A2E"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="FFE8792A"/>
+      <color rgb="FF1A9196"/>
       <sz val="9"/>
     </font>
     <font>
@@ -119,12 +119,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2D2D2D"/>
+        <fgColor rgb="FF085055"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEEF8F6"/>
+        <fgColor rgb="FFE4F5F6"/>
       </patternFill>
     </fill>
     <fill>
@@ -139,12 +139,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0A5F62"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8792A"/>
+        <fgColor rgb="FFCC6A2E"/>
       </patternFill>
     </fill>
     <fill>
@@ -154,22 +149,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF1E6"/>
+        <fgColor rgb="FFFFF4EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFCFE9E6"/>
+        <fgColor rgb="FFD9F0F1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF5F1EC"/>
+        <fgColor rgb="FFFFD0B3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFCE8D6"/>
+        <fgColor rgb="FF1A9196"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCEEEF"/>
       </patternFill>
     </fill>
   </fills>
@@ -183,21 +183,21 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9CEC0"/>
+        <color rgb="00CFE3E4"/>
       </left>
       <right style="thin">
-        <color rgb="00D9CEC0"/>
+        <color rgb="00CFE3E4"/>
       </right>
       <top style="thin">
-        <color rgb="00D9CEC0"/>
+        <color rgb="00CFE3E4"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9CEC0"/>
+        <color rgb="00CFE3E4"/>
       </bottom>
     </border>
     <border>
       <bottom style="thin">
-        <color rgb="00D9CEC0"/>
+        <color rgb="00CFE3E4"/>
       </bottom>
     </border>
     <border>
@@ -255,27 +255,27 @@
         <color rgb="000F868A"/>
       </left>
       <right style="thin">
-        <color rgb="00D9CEC0"/>
+        <color rgb="00CFE3E4"/>
       </right>
       <top style="thin">
-        <color rgb="00D9CEC0"/>
+        <color rgb="00CFE3E4"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9CEC0"/>
+        <color rgb="00CFE3E4"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9CEC0"/>
+        <color rgb="00CFE3E4"/>
       </left>
       <right style="medium">
         <color rgb="000F868A"/>
       </right>
       <top style="thin">
-        <color rgb="00D9CEC0"/>
+        <color rgb="00CFE3E4"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9CEC0"/>
+        <color rgb="00CFE3E4"/>
       </bottom>
     </border>
     <border>
@@ -283,7 +283,7 @@
         <color rgb="000F868A"/>
       </right>
       <bottom style="thin">
-        <color rgb="00D9CEC0"/>
+        <color rgb="00CFE3E4"/>
       </bottom>
     </border>
     <border>
@@ -320,7 +320,7 @@
   </cellStyleXfs>
   <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -345,15 +345,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -377,34 +377,52 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -419,25 +437,7 @@
     <xf numFmtId="0" fontId="10" fillId="10" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">

</xml_diff>